<commit_message>
chore: run 2026-03-23 16:21 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_23_03_2026.xlsx
+++ b/logs/Consolidado_23_03_2026.xlsx
@@ -8828,7 +8828,7 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>8197119</t>
+          <t>8197145</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
@@ -26555,7 +26555,7 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>8197119</t>
+          <t>8197145</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore: run 2026-03-23 17:41 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_23_03_2026.xlsx
+++ b/logs/Consolidado_23_03_2026.xlsx
@@ -8828,7 +8828,7 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>8197145</t>
+          <t>8197119</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
@@ -26555,7 +26555,7 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>8197145</t>
+          <t>8197119</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore: run 2026-03-23 22:41 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_23_03_2026.xlsx
+++ b/logs/Consolidado_23_03_2026.xlsx
@@ -676,10 +676,10 @@
         <v>78</v>
       </c>
       <c r="C4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -10804,40 +10804,40 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>23/03/2026</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>23/03/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Chamomile Brightening Blond Hair Conditioner
 Condicionador Camomila Brilho Cabelo Loiro
 200 ml</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/chamomile-brightening-blond-hair-conditioner-5870419.html</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr"/>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr"/>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>5870419</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>30%</t>
         </is>

</xml_diff>